<commit_message>
Réécriture de DataLoader pour inclure diet dans les table des consommateur. Création de df_energy
</commit_message>
<xml_diff>
--- a/example/GRAFS_data_example_N.xlsx
+++ b/example/GRAFS_data_example_N.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35CCB0E3-71B7-4792-A569-796BF685F0C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B580DB0-EDF2-4D66-9097-A18C4D6EED12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{F475FEA0-B9E5-4A03-9EDE-4A3E6C5C262C}"/>
+    <workbookView minimized="1" xWindow="2265" yWindow="-12000" windowWidth="14400" windowHeight="7275" xr2:uid="{F475FEA0-B9E5-4A03-9EDE-4A3E6C5C262C}"/>
   </bookViews>
   <sheets>
     <sheet name="Input data" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
Ajout d'un df energy et gestion flexible des infrastructures energétiques. Reste à mettre à jour la couche carbone. Mettre à jour l'exemple sur le carbone et la doc.
</commit_message>
<xml_diff>
--- a/example/GRAFS_data_example_N.xlsx
+++ b/example/GRAFS_data_example_N.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B580DB0-EDF2-4D66-9097-A18C4D6EED12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11D18537-3C3C-4CCF-87D2-7D18E69B6EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2265" yWindow="-12000" windowWidth="14400" windowHeight="7275" xr2:uid="{F475FEA0-B9E5-4A03-9EDE-4A3E6C5C262C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{F475FEA0-B9E5-4A03-9EDE-4A3E6C5C262C}"/>
   </bookViews>
   <sheets>
     <sheet name="Input data" sheetId="2" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="83">
   <si>
     <t>Area</t>
   </si>
@@ -294,6 +294,12 @@
   </si>
   <si>
     <t>Fishery ingestion per capita (kgN)</t>
+  </si>
+  <si>
+    <t>Bio_diet</t>
+  </si>
+  <si>
+    <t>Forage</t>
   </si>
 </sst>
 </file>
@@ -3829,7 +3835,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D80ABBC0-87F2-4F7A-9036-33771C52D9AC}">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -4208,6 +4214,17 @@
       </c>
       <c r="C34" t="s">
         <v>74</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>81</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>